<commit_message>
Upgrade video display in camera panel
</commit_message>
<xml_diff>
--- a/ros2_ws/src/flychams_bringup/config/Configuration-Test.xlsx
+++ b/ros2_ws/src/flychams_bringup/config/Configuration-Test.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="3"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="8"/>
   </bookViews>
   <sheets>
     <sheet name="Mission" sheetId="1" state="visible" r:id="rId3"/>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="691" uniqueCount="321">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="691" uniqueCount="320">
   <si>
     <t xml:space="preserve">GENERAL CONFIGURATION</t>
   </si>
@@ -953,9 +953,6 @@
   </si>
   <si>
     <t xml:space="preserve">Operational Conditions O1 (ultra-high-resolution camera)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">(7680x4320)</t>
   </si>
   <si>
     <t xml:space="preserve">CAM05</t>
@@ -2337,22 +2334,22 @@
         <v>2</v>
       </c>
       <c r="C2" s="20" t="s">
+        <v>310</v>
+      </c>
+      <c r="D2" s="20" t="s">
         <v>311</v>
       </c>
-      <c r="D2" s="20" t="s">
+      <c r="E2" s="20" t="s">
         <v>312</v>
       </c>
-      <c r="E2" s="20" t="s">
+      <c r="F2" s="20" t="s">
         <v>313</v>
       </c>
-      <c r="F2" s="20" t="s">
+      <c r="G2" s="20" t="s">
         <v>314</v>
       </c>
-      <c r="G2" s="20" t="s">
+      <c r="H2" s="20" t="s">
         <v>315</v>
-      </c>
-      <c r="H2" s="20" t="s">
-        <v>316</v>
       </c>
       <c r="I2" s="20" t="s">
         <v>290</v>
@@ -2371,28 +2368,28 @@
         <v>147</v>
       </c>
       <c r="B3" s="21" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="C3" s="21" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
       <c r="D3" s="21" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="E3" s="21" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
       <c r="F3" s="21" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="G3" s="21" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
       <c r="H3" s="21" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="I3" s="21" t="n">
         <v>0.4</v>
@@ -6013,7 +6010,7 @@
         <v>294</v>
       </c>
       <c r="D7" s="21" t="s">
-        <v>308</v>
+        <v>295</v>
       </c>
       <c r="E7" s="21" t="s">
         <v>296</v>
@@ -6040,16 +6037,16 @@
     </row>
     <row r="8" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="21" t="s">
+        <v>308</v>
+      </c>
+      <c r="B8" s="21" t="s">
         <v>309</v>
-      </c>
-      <c r="B8" s="21" t="s">
-        <v>310</v>
       </c>
       <c r="C8" s="21" t="s">
         <v>294</v>
       </c>
       <c r="D8" s="21" t="s">
-        <v>308</v>
+        <v>295</v>
       </c>
       <c r="E8" s="21" t="s">
         <v>296</v>

</xml_diff>